<commit_message>
Added a script to convert images to webp
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sdcr2613\Desktop\BS_PD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssamu\Desktop\Coding\alas-catalogo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B966A39E-4A24-477F-8BE2-105955C5D3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1043F075-EEE4-4D3C-A29F-67A9D99C60ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{D3EE13C3-C0F4-4078-9950-3F2F6B639038}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D3EE13C3-C0F4-4078-9950-3F2F6B639038}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="5" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="136">
   <si>
     <t>Product Image</t>
   </si>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t>Inspirado en la serenidad del mar, este anillo captura la esencia de lo natural con un diseño orgánico y elegante que evoca calma y libertad. \n\n**Cuidados**: Evitar agua salada y químicos. Limpiar con paño seco.</t>
+  </si>
+  <si>
+    <t>Anillo Curvas Abstractas</t>
   </si>
 </sst>
 </file>
@@ -3199,7 +3202,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -3515,16 +3518,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17A0122F-59D4-4637-BE6F-DD49479A8C39}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" style="3" customWidth="1"/>
-    <col min="4" max="11" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.88671875" customWidth="1"/>
+    <col min="2" max="2" width="36.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" style="3" customWidth="1"/>
+    <col min="4" max="11" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -3559,7 +3563,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -3594,7 +3598,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -3629,7 +3633,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -3664,7 +3668,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -3699,7 +3703,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -3734,7 +3738,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -3769,7 +3773,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -3804,7 +3808,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -3839,7 +3843,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -3874,7 +3878,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -3909,7 +3913,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -3944,7 +3948,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -3979,7 +3983,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -4014,7 +4018,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -4049,7 +4053,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
@@ -4084,7 +4088,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -4119,7 +4123,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
@@ -4154,7 +4158,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>26</v>
       </c>
@@ -4189,7 +4193,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -4224,7 +4228,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
@@ -4259,7 +4263,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -4294,7 +4298,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -4329,7 +4333,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>29</v>
       </c>
@@ -4364,7 +4368,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>30</v>
       </c>
@@ -4399,9 +4403,9 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>18</v>
+        <v>135</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>56</v>
@@ -4434,7 +4438,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>31</v>
       </c>
@@ -4469,7 +4473,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>32</v>
       </c>
@@ -4504,7 +4508,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
@@ -4539,7 +4543,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>33</v>
       </c>
@@ -4574,7 +4578,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>33</v>
       </c>
@@ -4609,7 +4613,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>34</v>
       </c>
@@ -4644,7 +4648,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>35</v>
       </c>
@@ -4679,7 +4683,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>35</v>
       </c>
@@ -4714,7 +4718,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>36</v>
       </c>
@@ -4749,7 +4753,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>37</v>
       </c>
@@ -4784,7 +4788,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
@@ -4820,7 +4824,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}"/>
+  <autoFilter ref="A1:K37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Anillo Corazón Asimétrico"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -4829,17 +4839,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03A83E87-90D2-4FFE-A6A7-E278883B4F92}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.42578125" customWidth="1"/>
-    <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.140625" customWidth="1"/>
-    <col min="4" max="4" width="14.42578125" style="3" customWidth="1"/>
-    <col min="5" max="12" width="14.42578125" customWidth="1"/>
+    <col min="1" max="1" width="14.44140625" customWidth="1"/>
+    <col min="2" max="2" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.109375" customWidth="1"/>
+    <col min="4" max="4" width="14.44140625" style="3" customWidth="1"/>
+    <col min="5" max="12" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4877,7 +4888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="79.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="79.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -4913,7 +4924,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -4949,7 +4960,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -4985,7 +4996,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -5021,7 +5032,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -5057,7 +5068,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -5093,7 +5104,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -5129,7 +5140,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -5165,7 +5176,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -5201,7 +5212,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -5237,7 +5248,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -5273,7 +5284,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -5309,7 +5320,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -5345,7 +5356,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>1</v>
       </c>
@@ -5381,7 +5392,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>1</v>
       </c>
@@ -5417,7 +5428,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>1</v>
       </c>
@@ -5453,7 +5464,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
@@ -5489,7 +5500,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -5525,7 +5536,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
@@ -5561,7 +5572,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>1</v>
       </c>
@@ -5597,7 +5608,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>1</v>
       </c>
@@ -5633,7 +5644,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>1</v>
       </c>
@@ -5669,7 +5680,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>1</v>
       </c>
@@ -5705,7 +5716,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>1</v>
       </c>
@@ -5741,7 +5752,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>1</v>
       </c>
@@ -5777,7 +5788,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
@@ -5813,7 +5824,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>1</v>
       </c>
@@ -5849,7 +5860,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>1</v>
       </c>
@@ -5885,7 +5896,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>1</v>
       </c>
@@ -5921,7 +5932,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>1</v>
       </c>
@@ -5957,7 +5968,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>1</v>
       </c>
@@ -5993,7 +6004,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>1</v>
       </c>
@@ -6029,7 +6040,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>1</v>
       </c>
@@ -6065,7 +6076,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>1</v>
       </c>
@@ -6101,7 +6112,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>1</v>
       </c>
@@ -6137,7 +6148,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>1</v>
       </c>
@@ -6173,17 +6184,23 @@
         <v>131</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="39" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:L37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}"/>
+  <autoFilter ref="A1:L37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="Anillo Corazón Asimétrico"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>

<commit_message>
feat: add ProductGallery component for responsive image display with thumbnails
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ssamu\Desktop\Coding\alas-catalogo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1043F075-EEE4-4D3C-A29F-67A9D99C60ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90EB2422-06EB-4577-BA1B-7F00D7C1E553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D3EE13C3-C0F4-4078-9950-3F2F6B639038}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D3EE13C3-C0F4-4078-9950-3F2F6B639038}"/>
   </bookViews>
   <sheets>
     <sheet name="products" sheetId="5" r:id="rId1"/>
@@ -3518,17 +3518,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17A0122F-59D4-4637-BE6F-DD49479A8C39}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="20.88671875" customWidth="1"/>
-    <col min="2" max="2" width="36.109375" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" style="3" customWidth="1"/>
-    <col min="4" max="11" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.42578125" style="3" customWidth="1"/>
+    <col min="4" max="11" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -3563,7 +3562,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>14</v>
       </c>
@@ -3598,7 +3597,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -3633,7 +3632,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>15</v>
       </c>
@@ -3668,7 +3667,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -3703,7 +3702,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -3738,7 +3737,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
@@ -3773,7 +3772,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>17</v>
       </c>
@@ -3808,7 +3807,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -3843,7 +3842,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -3878,7 +3877,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -3913,7 +3912,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -3948,7 +3947,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -3983,7 +3982,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
@@ -4018,7 +4017,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -4053,7 +4052,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>23</v>
       </c>
@@ -4088,7 +4087,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>24</v>
       </c>
@@ -4123,7 +4122,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>25</v>
       </c>
@@ -4158,7 +4157,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>26</v>
       </c>
@@ -4193,7 +4192,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -4228,7 +4227,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>28</v>
       </c>
@@ -4263,7 +4262,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>28</v>
       </c>
@@ -4298,7 +4297,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>29</v>
       </c>
@@ -4333,7 +4332,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>29</v>
       </c>
@@ -4368,7 +4367,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>30</v>
       </c>
@@ -4403,7 +4402,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>135</v>
       </c>
@@ -4438,7 +4437,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>31</v>
       </c>
@@ -4473,7 +4472,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>32</v>
       </c>
@@ -4508,7 +4507,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>32</v>
       </c>
@@ -4543,7 +4542,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>33</v>
       </c>
@@ -4578,7 +4577,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>33</v>
       </c>
@@ -4613,7 +4612,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>34</v>
       </c>
@@ -4648,7 +4647,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>35</v>
       </c>
@@ -4683,7 +4682,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>35</v>
       </c>
@@ -4718,7 +4717,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>36</v>
       </c>
@@ -4753,7 +4752,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>37</v>
       </c>
@@ -4788,7 +4787,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>38</v>
       </c>
@@ -4824,13 +4823,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Anillo Corazón Asimétrico"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
@@ -4841,16 +4834,16 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03A83E87-90D2-4FFE-A6A7-E278883B4F92}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:L47"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.44140625" customWidth="1"/>
-    <col min="2" max="2" width="36.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="36.109375" customWidth="1"/>
-    <col min="4" max="4" width="14.44140625" style="3" customWidth="1"/>
-    <col min="5" max="12" width="14.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="36.140625" customWidth="1"/>
+    <col min="4" max="4" width="14.42578125" style="3" customWidth="1"/>
+    <col min="5" max="12" width="14.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="13.8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4888,7 +4881,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="79.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="79.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -4924,7 +4917,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -4960,7 +4953,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -4996,7 +4989,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>1</v>
       </c>
@@ -5032,7 +5025,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -5068,7 +5061,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -5104,7 +5097,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -5140,7 +5133,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -5176,7 +5169,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -5212,7 +5205,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -5248,7 +5241,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>1</v>
       </c>
@@ -5284,7 +5277,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -5320,7 +5313,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -5356,7 +5349,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>1</v>
       </c>
@@ -5392,7 +5385,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>1</v>
       </c>
@@ -5428,7 +5421,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>1</v>
       </c>
@@ -5464,7 +5457,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>1</v>
       </c>
@@ -5500,7 +5493,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -5536,7 +5529,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>1</v>
       </c>
@@ -5572,7 +5565,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>1</v>
       </c>
@@ -5608,7 +5601,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>1</v>
       </c>
@@ -5644,7 +5637,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>1</v>
       </c>
@@ -5680,7 +5673,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>1</v>
       </c>
@@ -5716,7 +5709,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>1</v>
       </c>
@@ -5752,7 +5745,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>1</v>
       </c>
@@ -5788,7 +5781,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>1</v>
       </c>
@@ -5824,7 +5817,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>1</v>
       </c>
@@ -5860,7 +5853,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>1</v>
       </c>
@@ -5896,7 +5889,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>1</v>
       </c>
@@ -5932,7 +5925,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>1</v>
       </c>
@@ -5968,7 +5961,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>1</v>
       </c>
@@ -6004,7 +5997,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>1</v>
       </c>
@@ -6040,7 +6033,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>1</v>
       </c>
@@ -6076,7 +6069,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>1</v>
       </c>
@@ -6112,7 +6105,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>1</v>
       </c>
@@ -6148,7 +6141,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="80.099999999999994" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>1</v>
       </c>
@@ -6184,15 +6177,15 @@
         <v>131</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <autoFilter ref="A1:L37" xr:uid="{C7F39E25-AA98-49CF-A972-006AFA0C8782}">
     <filterColumn colId="1">

</xml_diff>